<commit_message>
Update coal warehouse and density catalog
</commit_message>
<xml_diff>
--- a/public/data/DS_kho_than_va_ty_khoi.xlsx
+++ b/public/data/DS_kho_than_va_ty_khoi.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TTCO_TonKho_App_Repo\public\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OSC\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{785F3197-2E85-4F7B-AABD-E035CC742C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A35D9A-9916-4A93-AAAD-714BD48C0750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dm_kho" sheetId="2" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="105">
   <si>
     <t>ten_kho</t>
   </si>
@@ -144,12 +144,6 @@
     <t>Cám đá</t>
   </si>
   <si>
-    <t>Bùn 3A</t>
-  </si>
-  <si>
-    <t>Bùn 3B</t>
-  </si>
-  <si>
     <t>Cám 1</t>
   </si>
   <si>
@@ -174,9 +168,6 @@
     <t>Cám 6a.1</t>
   </si>
   <si>
-    <t>Cám 6a.1(sấy)</t>
-  </si>
-  <si>
     <t>Cám 6a.14</t>
   </si>
   <si>
@@ -216,23 +207,159 @@
     <t>Kho 39</t>
   </si>
   <si>
-    <t>Cám 2</t>
-  </si>
-  <si>
     <t>Don vi quan ly</t>
   </si>
   <si>
     <t>Cám 5b.1</t>
+  </si>
+  <si>
+    <t>Cục xô 1c</t>
+  </si>
+  <si>
+    <t>Cám 1 / Cám 2a.1</t>
+  </si>
+  <si>
+    <t>Cám 5a.1 / Cám 5b.1 / Cám 6a.1</t>
+  </si>
+  <si>
+    <t>Cám 5a.1 / Cám 5b.1 / Cám 6a.1 / Cám 1</t>
+  </si>
+  <si>
+    <t>Kho 26</t>
+  </si>
+  <si>
+    <t>Kho 27</t>
+  </si>
+  <si>
+    <t>Kho 28</t>
+  </si>
+  <si>
+    <t>Kho 32</t>
+  </si>
+  <si>
+    <t>Kho 33</t>
+  </si>
+  <si>
+    <t>Kho 34</t>
+  </si>
+  <si>
+    <t>PX Lọc Sấy than</t>
+  </si>
+  <si>
+    <t>Kho 28-1</t>
+  </si>
+  <si>
+    <t>PX Tuyển than 3</t>
+  </si>
+  <si>
+    <t>PX Ô tô</t>
+  </si>
+  <si>
+    <t>Kho 35</t>
+  </si>
+  <si>
+    <t>Kho 36</t>
+  </si>
+  <si>
+    <t>Kho 37</t>
+  </si>
+  <si>
+    <t>Kho 38</t>
+  </si>
+  <si>
+    <t>Kho 40</t>
+  </si>
+  <si>
+    <t>Kho 1-T4</t>
+  </si>
+  <si>
+    <t>PX Tuyển than 4</t>
+  </si>
+  <si>
+    <t>Kho 2-T4</t>
+  </si>
+  <si>
+    <t>Kho 3-T4</t>
+  </si>
+  <si>
+    <t>Kho 4-T4</t>
+  </si>
+  <si>
+    <t>Kho 5-T4</t>
+  </si>
+  <si>
+    <t>Bùn tuyển 3A</t>
+  </si>
+  <si>
+    <t>Bùn tuyển 3A / Cám 6A.1 (sấy) / Cám 6b.1</t>
+  </si>
+  <si>
+    <t>Cám 6a.1 / Nhập khẩu</t>
+  </si>
+  <si>
+    <t>Nhập khẩu</t>
+  </si>
+  <si>
+    <t>Nhập khẩu / Bùn tuyển 3A</t>
+  </si>
+  <si>
+    <t>Cám đá / Nguyên khai</t>
+  </si>
+  <si>
+    <t>Nguyên khai / Cục don 8C</t>
+  </si>
+  <si>
+    <t>Cám 6a.1 / Cục don 8C</t>
+  </si>
+  <si>
+    <t>Bùn tuyển 3B</t>
+  </si>
+  <si>
+    <t>Cám 6A.1 (sấy)</t>
+  </si>
+  <si>
+    <t>Cám 4b.1</t>
+  </si>
+  <si>
+    <t>Cám 6a.1 / Cám 6a.14</t>
+  </si>
+  <si>
+    <t>Cám 5a.1 / Cám 5a.14</t>
+  </si>
+  <si>
+    <t>Nguyên khai / Cám đá / Cám 6A.1 (sấy)</t>
+  </si>
+  <si>
+    <t>Cám 3c.1</t>
+  </si>
+  <si>
+    <t>Cám 7A</t>
+  </si>
+  <si>
+    <t>Cám 7B</t>
+  </si>
+  <si>
+    <t>Cám 7C</t>
+  </si>
+  <si>
+    <t>Cám 8A</t>
+  </si>
+  <si>
+    <t>Cám 8B</t>
+  </si>
+  <si>
+    <t>Cám 8C</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -250,6 +377,10 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -292,11 +423,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -310,9 +442,17 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Bình thường" xfId="0" builtinId="0"/>
+    <cellStyle name="Dấu phẩy" xfId="2" builtinId="3"/>
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
   </cellStyles>
   <dxfs count="2">
@@ -366,7 +506,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DM_KHO" displayName="DM_KHO" ref="A1:E34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="DM_KHO" displayName="DM_KHO" ref="A1:E47">
   <tableColumns count="5">
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="ten_kho"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Don vi quan ly"/>
@@ -379,7 +519,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DM_TY_KHOI" displayName="DM_TY_KHOI" ref="A1:C23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DM_TY_KHOI" displayName="DM_TY_KHOI" ref="A1:C31">
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="stt"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="chung_loai"/>
@@ -538,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:Y85"/>
+  <dimension ref="A1:Y97"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -551,13 +691,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -588,15 +728,17 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="2">
-        <v>48.3</v>
-      </c>
-      <c r="D2" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E2" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C2" s="5">
+        <v>50.618279569892472</v>
+      </c>
+      <c r="D2" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
@@ -623,15 +765,17 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C3" s="2">
-        <v>78</v>
-      </c>
-      <c r="D3" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E3" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C3" s="5">
+        <v>76.666666666666657</v>
+      </c>
+      <c r="D3" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
@@ -658,15 +802,17 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="2">
-        <v>74</v>
-      </c>
-      <c r="D4" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E4" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C4" s="5">
+        <v>75.053763440860209</v>
+      </c>
+      <c r="D4" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
@@ -693,15 +839,17 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="2">
-        <v>84</v>
-      </c>
-      <c r="D5" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E5" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C5" s="5">
+        <v>85.107526881720418</v>
+      </c>
+      <c r="D5" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
@@ -728,15 +876,17 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C6" s="2">
-        <v>75.5</v>
-      </c>
-      <c r="D6" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E6" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C6" s="5">
+        <v>75.134408602150529</v>
+      </c>
+      <c r="D6" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
@@ -763,15 +913,17 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C7" s="2">
-        <v>48</v>
-      </c>
-      <c r="D7" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E7" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C7" s="5">
+        <v>48.198924731182792</v>
+      </c>
+      <c r="D7" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -798,15 +950,17 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="2">
-        <v>147.9</v>
-      </c>
-      <c r="D8" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E8" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C8" s="5">
+        <v>161.93548387096774</v>
+      </c>
+      <c r="D8" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
@@ -833,15 +987,17 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C9" s="2">
-        <v>182</v>
-      </c>
-      <c r="D9" s="2">
-        <v>36.5</v>
-      </c>
-      <c r="E9" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C9" s="5">
+        <v>167.44623655913978</v>
+      </c>
+      <c r="D9" s="5">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -868,16 +1024,16 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" s="2">
-        <v>167.7</v>
-      </c>
-      <c r="D10" s="2">
-        <v>40.9</v>
+        <v>53</v>
+      </c>
+      <c r="C10" s="5">
+        <v>229.70101309612059</v>
+      </c>
+      <c r="D10" s="5">
+        <v>40.47</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>45</v>
+        <v>95</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -902,19 +1058,19 @@
     </row>
     <row r="11" spans="1:25">
       <c r="A11" s="2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C11" s="2">
-        <v>40.700000000000003</v>
-      </c>
-      <c r="D11" s="2">
-        <v>40.9</v>
+        <v>53</v>
+      </c>
+      <c r="C11" s="5">
+        <v>192.76006918705215</v>
+      </c>
+      <c r="D11" s="5">
+        <v>40.47</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -939,19 +1095,19 @@
     </row>
     <row r="12" spans="1:25">
       <c r="A12" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="2">
-        <v>46.3</v>
-      </c>
-      <c r="D12" s="2">
-        <v>40.9</v>
+        <v>53</v>
+      </c>
+      <c r="C12" s="5">
+        <v>141.19100568322213</v>
+      </c>
+      <c r="D12" s="5">
+        <v>40.47</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -976,19 +1132,19 @@
     </row>
     <row r="13" spans="1:25">
       <c r="A13" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" s="2">
-        <v>131.84</v>
-      </c>
-      <c r="D13" s="2">
-        <v>40.9</v>
+        <v>53</v>
+      </c>
+      <c r="C13" s="5">
+        <v>97.776130467012607</v>
+      </c>
+      <c r="D13" s="5">
+        <v>40.47</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1013,18 +1169,20 @@
     </row>
     <row r="14" spans="1:25">
       <c r="A14" s="2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C14" s="2">
-        <v>145.1</v>
-      </c>
-      <c r="D14" s="2">
-        <v>40.9</v>
-      </c>
-      <c r="E14" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C14" s="5">
+        <v>69.360019767729185</v>
+      </c>
+      <c r="D14" s="5">
+        <v>40.47</v>
+      </c>
+      <c r="E14" t="s">
+        <v>38</v>
+      </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
@@ -1048,18 +1206,20 @@
     </row>
     <row r="15" spans="1:25">
       <c r="A15" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C15" s="2">
-        <v>93.4</v>
-      </c>
-      <c r="D15" s="2">
-        <v>40.9</v>
-      </c>
-      <c r="E15" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C15" s="5">
+        <v>68.668149246355327</v>
+      </c>
+      <c r="D15" s="5">
+        <v>40.47</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
@@ -1083,18 +1243,20 @@
     </row>
     <row r="16" spans="1:25">
       <c r="A16" s="2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" s="2">
-        <v>69.2</v>
-      </c>
-      <c r="D16" s="2">
-        <v>40.9</v>
-      </c>
-      <c r="E16" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C16" s="5">
+        <v>130.9612058314801</v>
+      </c>
+      <c r="D16" s="5">
+        <v>40.47</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -1118,18 +1280,20 @@
     </row>
     <row r="17" spans="1:25">
       <c r="A17" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="2">
-        <v>0</v>
-      </c>
-      <c r="D17" s="2">
-        <v>40.9</v>
-      </c>
-      <c r="E17" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C17" s="5">
+        <v>114.22330097087378</v>
+      </c>
+      <c r="D17" s="5">
+        <v>41.2</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -1153,18 +1317,20 @@
     </row>
     <row r="18" spans="1:25">
       <c r="A18" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C18" s="2">
-        <v>198.5</v>
-      </c>
-      <c r="D18" s="2">
-        <v>40.9</v>
-      </c>
-      <c r="E18" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C18" s="5">
+        <v>286.09223300970871</v>
+      </c>
+      <c r="D18" s="5">
+        <v>41.2</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -1188,18 +1354,20 @@
     </row>
     <row r="19" spans="1:25">
       <c r="A19" s="2" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C19" s="2">
-        <v>108</v>
-      </c>
-      <c r="D19" s="2">
-        <v>41</v>
-      </c>
-      <c r="E19" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C19" s="5">
+        <v>81.626213592233</v>
+      </c>
+      <c r="D19" s="5">
+        <v>41.2</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -1223,19 +1391,19 @@
     </row>
     <row r="20" spans="1:25">
       <c r="A20" s="2" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C20" s="2">
-        <v>104</v>
-      </c>
-      <c r="D20" s="2">
-        <v>41</v>
+        <v>53</v>
+      </c>
+      <c r="C20" s="5">
+        <v>55.194174757281552</v>
+      </c>
+      <c r="D20" s="5">
+        <v>41.2</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>60</v>
+        <v>39</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1260,19 +1428,19 @@
     </row>
     <row r="21" spans="1:25">
       <c r="A21" s="2" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="2">
-        <v>205.6</v>
-      </c>
-      <c r="D21" s="2">
-        <v>41</v>
+        <v>53</v>
+      </c>
+      <c r="C21" s="5">
+        <v>217.40291262135921</v>
+      </c>
+      <c r="D21" s="5">
+        <v>41.2</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1297,18 +1465,20 @@
     </row>
     <row r="22" spans="1:25">
       <c r="A22" s="2" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C22" s="2">
-        <v>63.7</v>
-      </c>
-      <c r="D22" s="2">
-        <v>41</v>
-      </c>
-      <c r="E22" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C22" s="5">
+        <v>66.50485436893203</v>
+      </c>
+      <c r="D22" s="5">
+        <v>41.2</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -1332,18 +1502,20 @@
     </row>
     <row r="23" spans="1:25">
       <c r="A23" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C23" s="2">
-        <v>39</v>
-      </c>
-      <c r="D23" s="2">
-        <v>41</v>
-      </c>
-      <c r="E23" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C23" s="5">
+        <v>101.96601941747572</v>
+      </c>
+      <c r="D23" s="5">
+        <v>41.2</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>62</v>
+      </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -1367,18 +1539,20 @@
     </row>
     <row r="24" spans="1:25">
       <c r="A24" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C24" s="2">
-        <v>233</v>
-      </c>
-      <c r="D24" s="2">
-        <v>41</v>
-      </c>
-      <c r="E24" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C24" s="5">
+        <v>132.27011494252875</v>
+      </c>
+      <c r="D24" s="5">
+        <v>34.799999999999997</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -1402,19 +1576,19 @@
     </row>
     <row r="25" spans="1:25">
       <c r="A25" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C25" s="2">
-        <v>55</v>
-      </c>
-      <c r="D25" s="2">
-        <v>41</v>
+        <v>53</v>
+      </c>
+      <c r="C25" s="5">
+        <v>144.10919540229887</v>
+      </c>
+      <c r="D25" s="5">
+        <v>34.799999999999997</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1439,19 +1613,19 @@
     </row>
     <row r="26" spans="1:25">
       <c r="A26" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="2">
-        <v>55</v>
-      </c>
-      <c r="D26" s="2">
-        <v>41</v>
+        <v>53</v>
+      </c>
+      <c r="C26" s="5">
+        <v>134.77011494252875</v>
+      </c>
+      <c r="D26" s="5">
+        <v>34.799999999999997</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1476,19 +1650,19 @@
     </row>
     <row r="27" spans="1:25">
       <c r="A27" s="2" t="s">
-        <v>22</v>
+        <v>63</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C27" s="2">
-        <v>56</v>
-      </c>
-      <c r="D27" s="2">
-        <v>41</v>
+        <v>69</v>
+      </c>
+      <c r="C27" s="6">
+        <v>92.205542725173203</v>
+      </c>
+      <c r="D27" s="6">
+        <v>34.64</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1513,18 +1687,20 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="2" t="s">
-        <v>23</v>
+        <v>64</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C28" s="2">
-        <v>60</v>
-      </c>
-      <c r="D28" s="2">
-        <v>41</v>
-      </c>
-      <c r="E28" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="C28" s="6">
+        <v>109.06478578892371</v>
+      </c>
+      <c r="D28" s="6">
+        <v>38.28</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -1548,18 +1724,20 @@
     </row>
     <row r="29" spans="1:25">
       <c r="A29" s="2" t="s">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C29" s="2">
-        <v>116</v>
-      </c>
-      <c r="D29" s="2">
-        <v>35.200000000000003</v>
-      </c>
-      <c r="E29" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="C29" s="6">
+        <v>108.76259798432251</v>
+      </c>
+      <c r="D29" s="6">
+        <v>35.72</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -1583,18 +1761,20 @@
     </row>
     <row r="30" spans="1:25">
       <c r="A30" s="2" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" s="2">
-        <v>144</v>
-      </c>
-      <c r="D30" s="2">
-        <v>35.200000000000003</v>
-      </c>
-      <c r="E30" s="2"/>
+        <v>69</v>
+      </c>
+      <c r="C30" s="6">
+        <v>108.34141610087293</v>
+      </c>
+      <c r="D30" s="6">
+        <v>41.24</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -1618,18 +1798,20 @@
     </row>
     <row r="31" spans="1:25">
       <c r="A31" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="2">
-        <v>122</v>
-      </c>
-      <c r="D31" s="2">
-        <v>35.200000000000003</v>
-      </c>
-      <c r="E31" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C31" s="6">
+        <v>194.60619062212686</v>
+      </c>
+      <c r="D31" s="6">
+        <v>32.630000000000003</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -1653,18 +1835,20 @@
     </row>
     <row r="32" spans="1:25">
       <c r="A32" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C32" s="2">
-        <v>127.7</v>
-      </c>
-      <c r="D32" s="2">
-        <v>31.8</v>
-      </c>
-      <c r="E32" s="2"/>
+        <v>53</v>
+      </c>
+      <c r="C32" s="6">
+        <v>118.97027275513331</v>
+      </c>
+      <c r="D32" s="6">
+        <v>32.630000000000003</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
@@ -1688,18 +1872,20 @@
     </row>
     <row r="33" spans="1:25">
       <c r="A33" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="2">
-        <v>143</v>
-      </c>
-      <c r="D33" s="2">
-        <v>31.8</v>
-      </c>
-      <c r="E33" s="2"/>
+        <v>30</v>
+      </c>
+      <c r="C33" s="5">
+        <v>189.28865696237298</v>
+      </c>
+      <c r="D33" s="5">
+        <v>36.409999999999997</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>31</v>
+      </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -1723,19 +1909,19 @@
     </row>
     <row r="34" spans="1:25">
       <c r="A34" s="2" t="s">
-        <v>29</v>
+        <v>66</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C34" s="2">
-        <v>190</v>
-      </c>
-      <c r="D34" s="2">
-        <v>35.799999999999997</v>
+        <v>71</v>
+      </c>
+      <c r="C34" s="6">
+        <v>110</v>
+      </c>
+      <c r="D34" s="6">
+        <v>60</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>31</v>
+        <v>97</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1760,18 +1946,20 @@
     </row>
     <row r="35" spans="1:25">
       <c r="A35" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="C35" s="2">
-        <v>214</v>
-      </c>
-      <c r="D35" s="2">
-        <v>32.049999999999997</v>
-      </c>
-      <c r="E35" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C35" s="6">
+        <v>227.33438842414651</v>
+      </c>
+      <c r="D35" s="6">
+        <v>44.23</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
@@ -1794,11 +1982,21 @@
       <c r="Y35" s="2"/>
     </row>
     <row r="36" spans="1:25">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="A36" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="6">
+        <v>150.87445346658336</v>
+      </c>
+      <c r="D36" s="6">
+        <v>64.040000000000006</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -1821,11 +2019,21 @@
       <c r="Y36" s="2"/>
     </row>
     <row r="37" spans="1:25">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+      <c r="A37" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="6">
+        <v>292.70999999999998</v>
+      </c>
+      <c r="D37" s="6">
+        <v>138.3519524443989</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -1848,11 +2056,21 @@
       <c r="Y37" s="2"/>
     </row>
     <row r="38" spans="1:25">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="A38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C38" s="6">
+        <v>191.39066863808117</v>
+      </c>
+      <c r="D38" s="6">
+        <v>121.74</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -1875,11 +2093,21 @@
       <c r="Y38" s="2"/>
     </row>
     <row r="39" spans="1:25">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="A39" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C39" s="6">
+        <v>189.93333333333334</v>
+      </c>
+      <c r="D39" s="6">
+        <v>75</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>84</v>
+      </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -1902,11 +2130,21 @@
       <c r="Y39" s="2"/>
     </row>
     <row r="40" spans="1:25">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="A40" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="6">
+        <v>210.89831909616976</v>
+      </c>
+      <c r="D40" s="6">
+        <v>145.16</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>89</v>
+      </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
@@ -1929,11 +2167,21 @@
       <c r="Y40" s="2"/>
     </row>
     <row r="41" spans="1:25">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
+      <c r="A41" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="6">
+        <v>214.11</v>
+      </c>
+      <c r="D41" s="6">
+        <v>39.29288683387044</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
@@ -1956,11 +2204,21 @@
       <c r="Y41" s="2"/>
     </row>
     <row r="42" spans="1:25">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="A42" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="C42" s="6">
+        <v>182.01</v>
+      </c>
+      <c r="D42" s="6">
+        <v>32.531179605516179</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -1983,11 +2241,21 @@
       <c r="Y42" s="2"/>
     </row>
     <row r="43" spans="1:25">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
+      <c r="A43" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="5">
+        <v>267.51</v>
+      </c>
+      <c r="D43" s="5">
+        <v>96.830025045792681</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
@@ -2010,11 +2278,21 @@
       <c r="Y43" s="2"/>
     </row>
     <row r="44" spans="1:25">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="A44" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="5">
+        <v>148.08000000000001</v>
+      </c>
+      <c r="D44" s="5">
+        <v>87.655321447866015</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -2037,65 +2315,55 @@
       <c r="Y44" s="2"/>
     </row>
     <row r="45" spans="1:25">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2"/>
-      <c r="U45" s="2"/>
-      <c r="V45" s="2"/>
-      <c r="W45" s="2"/>
-      <c r="X45" s="2"/>
-      <c r="Y45" s="2"/>
+      <c r="A45" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="7">
+        <v>192.38</v>
+      </c>
+      <c r="D45" s="7">
+        <v>37.010084208337666</v>
+      </c>
+      <c r="E45" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="46" spans="1:25">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
-      <c r="H46" s="2"/>
-      <c r="I46" s="2"/>
-      <c r="J46" s="2"/>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
-      <c r="S46" s="2"/>
-      <c r="T46" s="2"/>
-      <c r="U46" s="2"/>
-      <c r="V46" s="2"/>
-      <c r="W46" s="2"/>
-      <c r="X46" s="2"/>
-      <c r="Y46" s="2"/>
+      <c r="A46" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="6">
+        <v>72.95</v>
+      </c>
+      <c r="D46" s="6">
+        <v>60.137080191912268</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="47" spans="1:25">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
+      <c r="A47" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="6">
+        <v>151.69999999999999</v>
+      </c>
+      <c r="D47" s="6">
+        <v>45.484508899143052</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
@@ -3143,7 +3411,312 @@
       <c r="X85" s="2"/>
       <c r="Y85" s="2"/>
     </row>
+    <row r="86" spans="1:25">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
+      <c r="L86" s="2"/>
+      <c r="M86" s="2"/>
+      <c r="N86" s="2"/>
+      <c r="O86" s="2"/>
+      <c r="P86" s="2"/>
+      <c r="Q86" s="2"/>
+      <c r="R86" s="2"/>
+      <c r="S86" s="2"/>
+      <c r="T86" s="2"/>
+      <c r="U86" s="2"/>
+      <c r="V86" s="2"/>
+      <c r="W86" s="2"/>
+      <c r="X86" s="2"/>
+      <c r="Y86" s="2"/>
+    </row>
+    <row r="87" spans="1:25">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="2"/>
+      <c r="K87" s="2"/>
+      <c r="L87" s="2"/>
+      <c r="M87" s="2"/>
+      <c r="N87" s="2"/>
+      <c r="O87" s="2"/>
+      <c r="P87" s="2"/>
+      <c r="Q87" s="2"/>
+      <c r="R87" s="2"/>
+      <c r="S87" s="2"/>
+      <c r="T87" s="2"/>
+      <c r="U87" s="2"/>
+      <c r="V87" s="2"/>
+      <c r="W87" s="2"/>
+      <c r="X87" s="2"/>
+      <c r="Y87" s="2"/>
+    </row>
+    <row r="88" spans="1:25">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
+      <c r="L88" s="2"/>
+      <c r="M88" s="2"/>
+      <c r="N88" s="2"/>
+      <c r="O88" s="2"/>
+      <c r="P88" s="2"/>
+      <c r="Q88" s="2"/>
+      <c r="R88" s="2"/>
+      <c r="S88" s="2"/>
+      <c r="T88" s="2"/>
+      <c r="U88" s="2"/>
+      <c r="V88" s="2"/>
+      <c r="W88" s="2"/>
+      <c r="X88" s="2"/>
+      <c r="Y88" s="2"/>
+    </row>
+    <row r="89" spans="1:25">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
+      <c r="I89" s="2"/>
+      <c r="J89" s="2"/>
+      <c r="K89" s="2"/>
+      <c r="L89" s="2"/>
+      <c r="M89" s="2"/>
+      <c r="N89" s="2"/>
+      <c r="O89" s="2"/>
+      <c r="P89" s="2"/>
+      <c r="Q89" s="2"/>
+      <c r="R89" s="2"/>
+      <c r="S89" s="2"/>
+      <c r="T89" s="2"/>
+      <c r="U89" s="2"/>
+      <c r="V89" s="2"/>
+      <c r="W89" s="2"/>
+      <c r="X89" s="2"/>
+      <c r="Y89" s="2"/>
+    </row>
+    <row r="90" spans="1:25">
+      <c r="A90" s="2"/>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="2"/>
+      <c r="E90" s="2"/>
+      <c r="F90" s="2"/>
+      <c r="G90" s="2"/>
+      <c r="H90" s="2"/>
+      <c r="I90" s="2"/>
+      <c r="J90" s="2"/>
+      <c r="K90" s="2"/>
+      <c r="L90" s="2"/>
+      <c r="M90" s="2"/>
+      <c r="N90" s="2"/>
+      <c r="O90" s="2"/>
+      <c r="P90" s="2"/>
+      <c r="Q90" s="2"/>
+      <c r="R90" s="2"/>
+      <c r="S90" s="2"/>
+      <c r="T90" s="2"/>
+      <c r="U90" s="2"/>
+      <c r="V90" s="2"/>
+      <c r="W90" s="2"/>
+      <c r="X90" s="2"/>
+      <c r="Y90" s="2"/>
+    </row>
+    <row r="91" spans="1:25">
+      <c r="A91" s="2"/>
+      <c r="B91" s="2"/>
+      <c r="C91" s="2"/>
+      <c r="D91" s="2"/>
+      <c r="E91" s="2"/>
+      <c r="F91" s="2"/>
+      <c r="G91" s="2"/>
+      <c r="H91" s="2"/>
+      <c r="I91" s="2"/>
+      <c r="J91" s="2"/>
+      <c r="K91" s="2"/>
+      <c r="L91" s="2"/>
+      <c r="M91" s="2"/>
+      <c r="N91" s="2"/>
+      <c r="O91" s="2"/>
+      <c r="P91" s="2"/>
+      <c r="Q91" s="2"/>
+      <c r="R91" s="2"/>
+      <c r="S91" s="2"/>
+      <c r="T91" s="2"/>
+      <c r="U91" s="2"/>
+      <c r="V91" s="2"/>
+      <c r="W91" s="2"/>
+      <c r="X91" s="2"/>
+      <c r="Y91" s="2"/>
+    </row>
+    <row r="92" spans="1:25">
+      <c r="A92" s="2"/>
+      <c r="B92" s="2"/>
+      <c r="C92" s="2"/>
+      <c r="D92" s="2"/>
+      <c r="E92" s="2"/>
+      <c r="F92" s="2"/>
+      <c r="G92" s="2"/>
+      <c r="H92" s="2"/>
+      <c r="I92" s="2"/>
+      <c r="J92" s="2"/>
+      <c r="K92" s="2"/>
+      <c r="L92" s="2"/>
+      <c r="M92" s="2"/>
+      <c r="N92" s="2"/>
+      <c r="O92" s="2"/>
+      <c r="P92" s="2"/>
+      <c r="Q92" s="2"/>
+      <c r="R92" s="2"/>
+      <c r="S92" s="2"/>
+      <c r="T92" s="2"/>
+      <c r="U92" s="2"/>
+      <c r="V92" s="2"/>
+      <c r="W92" s="2"/>
+      <c r="X92" s="2"/>
+      <c r="Y92" s="2"/>
+    </row>
+    <row r="93" spans="1:25">
+      <c r="A93" s="2"/>
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
+      <c r="H93" s="2"/>
+      <c r="I93" s="2"/>
+      <c r="J93" s="2"/>
+      <c r="K93" s="2"/>
+      <c r="L93" s="2"/>
+      <c r="M93" s="2"/>
+      <c r="N93" s="2"/>
+      <c r="O93" s="2"/>
+      <c r="P93" s="2"/>
+      <c r="Q93" s="2"/>
+      <c r="R93" s="2"/>
+      <c r="S93" s="2"/>
+      <c r="T93" s="2"/>
+      <c r="U93" s="2"/>
+      <c r="V93" s="2"/>
+      <c r="W93" s="2"/>
+      <c r="X93" s="2"/>
+      <c r="Y93" s="2"/>
+    </row>
+    <row r="94" spans="1:25">
+      <c r="A94" s="2"/>
+      <c r="B94" s="2"/>
+      <c r="C94" s="2"/>
+      <c r="D94" s="2"/>
+      <c r="E94" s="2"/>
+      <c r="F94" s="2"/>
+      <c r="G94" s="2"/>
+      <c r="H94" s="2"/>
+      <c r="I94" s="2"/>
+      <c r="J94" s="2"/>
+      <c r="K94" s="2"/>
+      <c r="L94" s="2"/>
+      <c r="M94" s="2"/>
+      <c r="N94" s="2"/>
+      <c r="O94" s="2"/>
+      <c r="P94" s="2"/>
+      <c r="Q94" s="2"/>
+      <c r="R94" s="2"/>
+      <c r="S94" s="2"/>
+      <c r="T94" s="2"/>
+      <c r="U94" s="2"/>
+      <c r="V94" s="2"/>
+      <c r="W94" s="2"/>
+      <c r="X94" s="2"/>
+      <c r="Y94" s="2"/>
+    </row>
+    <row r="95" spans="1:25">
+      <c r="A95" s="2"/>
+      <c r="B95" s="2"/>
+      <c r="C95" s="2"/>
+      <c r="D95" s="2"/>
+      <c r="E95" s="2"/>
+      <c r="F95" s="2"/>
+      <c r="G95" s="2"/>
+      <c r="H95" s="2"/>
+      <c r="I95" s="2"/>
+      <c r="J95" s="2"/>
+      <c r="K95" s="2"/>
+      <c r="L95" s="2"/>
+      <c r="M95" s="2"/>
+      <c r="N95" s="2"/>
+      <c r="O95" s="2"/>
+      <c r="P95" s="2"/>
+      <c r="Q95" s="2"/>
+      <c r="R95" s="2"/>
+      <c r="S95" s="2"/>
+      <c r="T95" s="2"/>
+      <c r="U95" s="2"/>
+      <c r="V95" s="2"/>
+      <c r="W95" s="2"/>
+      <c r="X95" s="2"/>
+      <c r="Y95" s="2"/>
+    </row>
+    <row r="96" spans="1:25">
+      <c r="A96" s="2"/>
+      <c r="B96" s="2"/>
+      <c r="C96" s="2"/>
+      <c r="D96" s="2"/>
+      <c r="E96" s="2"/>
+      <c r="F96" s="2"/>
+      <c r="G96" s="2"/>
+      <c r="H96" s="2"/>
+      <c r="I96" s="2"/>
+      <c r="J96" s="2"/>
+      <c r="K96" s="2"/>
+      <c r="L96" s="2"/>
+      <c r="M96" s="2"/>
+      <c r="N96" s="2"/>
+      <c r="O96" s="2"/>
+      <c r="P96" s="2"/>
+      <c r="Q96" s="2"/>
+      <c r="R96" s="2"/>
+      <c r="S96" s="2"/>
+      <c r="T96" s="2"/>
+      <c r="U96" s="2"/>
+      <c r="V96" s="2"/>
+      <c r="W96" s="2"/>
+      <c r="X96" s="2"/>
+      <c r="Y96" s="2"/>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97" s="2"/>
+      <c r="B97" s="2"/>
+      <c r="C97" s="2"/>
+      <c r="D97" s="2"/>
+      <c r="E97" s="2"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
@@ -3154,7 +3727,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:Z81"/>
+  <dimension ref="A1:Z89"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -3201,10 +3774,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="C2" s="3">
-        <v>1.3766666666666667</v>
+        <v>0.85117120418848147</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
@@ -3235,10 +3808,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="C3" s="3">
-        <v>1.2583689423076949</v>
+        <v>0.87113298429319397</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -3269,10 +3842,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C4" s="3">
-        <v>0.97824999999999995</v>
+        <v>0.87776293193717259</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
@@ -3303,7 +3876,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C5" s="3">
         <v>0.90840251366120195</v>
@@ -3337,7 +3910,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C6" s="3">
         <v>0.92027049180327902</v>
@@ -3371,7 +3944,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C7" s="3">
         <v>0.93945989071038305</v>
@@ -3405,7 +3978,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C8" s="3">
         <v>0.97699038251366144</v>
@@ -3439,10 +4012,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>42</v>
+        <v>98</v>
       </c>
       <c r="C9" s="3">
-        <v>1.01316721311475</v>
+        <v>0.98199999999999998</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
@@ -3473,10 +4046,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C10" s="3">
-        <v>1.1045441530054649</v>
+        <v>1.01316721311475</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -3507,9 +4080,11 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="3"/>
+        <v>94</v>
+      </c>
+      <c r="C11" s="3">
+        <v>1.01</v>
+      </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -3539,10 +4114,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C12" s="3">
-        <v>1.0953590163934399</v>
+        <v>1.1045441530054649</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -3573,10 +4148,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C13" s="3">
-        <v>1.1842624043715826</v>
+        <v>1.125</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -3607,10 +4182,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C14" s="3">
-        <v>1.1512852459016401</v>
+        <v>1.0953590163934399</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -3641,10 +4216,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C15" s="3">
-        <v>1.1783234972677601</v>
+        <v>1.1842624043715826</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -3675,10 +4250,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="C16" s="3">
-        <v>1.2069924590163925</v>
+        <v>1.1512852459016401</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -3709,10 +4284,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C17" s="3">
-        <v>0.85117120418848147</v>
+        <v>1.1783234972677601</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -3743,10 +4318,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C18" s="3">
-        <v>0.87113298429319397</v>
+        <v>1.2069924590163925</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
@@ -3780,7 +4355,7 @@
         <v>51</v>
       </c>
       <c r="C19" s="3">
-        <v>0.87776293193717259</v>
+        <v>1.22525</v>
       </c>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
@@ -3811,10 +4386,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C20" s="3">
-        <v>1.2562172631578901</v>
+        <v>0.93252816753926737</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -3845,10 +4420,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="C21" s="3">
-        <v>0.93252816753926737</v>
+        <v>1.2562172631578901</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -3879,10 +4454,10 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="C22" s="3">
-        <v>1.22525</v>
+        <v>1.2350000000000001</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -3913,10 +4488,10 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="C23" s="3">
-        <v>1.5920000000000001</v>
+        <v>1.26</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -3943,9 +4518,15 @@
       <c r="Z23" s="2"/>
     </row>
     <row r="24" spans="1:26">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C24" s="3">
+        <v>1.2649999999999999</v>
+      </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -3971,9 +4552,15 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" spans="1:26">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C25" s="3">
+        <v>1.3049999999999999</v>
+      </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
@@ -3999,9 +4586,15 @@
       <c r="Z25" s="2"/>
     </row>
     <row r="26" spans="1:26">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
-      <c r="C26" s="2"/>
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C26" s="3">
+        <v>1.33</v>
+      </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
@@ -4027,9 +4620,15 @@
       <c r="Z26" s="2"/>
     </row>
     <row r="27" spans="1:26">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="2"/>
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C27" s="3">
+        <v>1.4019999999999999</v>
+      </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -4055,9 +4654,15 @@
       <c r="Z27" s="2"/>
     </row>
     <row r="28" spans="1:26">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="3">
+        <v>1.3766666666666667</v>
+      </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
@@ -4083,9 +4688,15 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29" spans="1:26">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="2"/>
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C29" s="3">
+        <v>1.2583689423076949</v>
+      </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -4111,9 +4722,15 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30" spans="1:26">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0.97824999999999995</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
@@ -4139,9 +4756,15 @@
       <c r="Z30" s="2"/>
     </row>
     <row r="31" spans="1:26">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C31" s="3">
+        <v>1.5920000000000001</v>
+      </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
@@ -5566,6 +6189,230 @@
       <c r="Y81" s="2"/>
       <c r="Z81" s="2"/>
     </row>
+    <row r="82" spans="1:26">
+      <c r="A82" s="2"/>
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+      <c r="H82" s="2"/>
+      <c r="I82" s="2"/>
+      <c r="J82" s="2"/>
+      <c r="K82" s="2"/>
+      <c r="L82" s="2"/>
+      <c r="M82" s="2"/>
+      <c r="N82" s="2"/>
+      <c r="O82" s="2"/>
+      <c r="P82" s="2"/>
+      <c r="Q82" s="2"/>
+      <c r="R82" s="2"/>
+      <c r="S82" s="2"/>
+      <c r="T82" s="2"/>
+      <c r="U82" s="2"/>
+      <c r="V82" s="2"/>
+      <c r="W82" s="2"/>
+      <c r="X82" s="2"/>
+      <c r="Y82" s="2"/>
+      <c r="Z82" s="2"/>
+    </row>
+    <row r="83" spans="1:26">
+      <c r="A83" s="2"/>
+      <c r="B83" s="2"/>
+      <c r="C83" s="2"/>
+      <c r="D83" s="2"/>
+      <c r="E83" s="2"/>
+      <c r="F83" s="2"/>
+      <c r="G83" s="2"/>
+      <c r="H83" s="2"/>
+      <c r="I83" s="2"/>
+      <c r="J83" s="2"/>
+      <c r="K83" s="2"/>
+      <c r="L83" s="2"/>
+      <c r="M83" s="2"/>
+      <c r="N83" s="2"/>
+      <c r="O83" s="2"/>
+      <c r="P83" s="2"/>
+      <c r="Q83" s="2"/>
+      <c r="R83" s="2"/>
+      <c r="S83" s="2"/>
+      <c r="T83" s="2"/>
+      <c r="U83" s="2"/>
+      <c r="V83" s="2"/>
+      <c r="W83" s="2"/>
+      <c r="X83" s="2"/>
+      <c r="Y83" s="2"/>
+      <c r="Z83" s="2"/>
+    </row>
+    <row r="84" spans="1:26">
+      <c r="A84" s="2"/>
+      <c r="B84" s="2"/>
+      <c r="C84" s="2"/>
+      <c r="D84" s="2"/>
+      <c r="E84" s="2"/>
+      <c r="F84" s="2"/>
+      <c r="G84" s="2"/>
+      <c r="H84" s="2"/>
+      <c r="I84" s="2"/>
+      <c r="J84" s="2"/>
+      <c r="K84" s="2"/>
+      <c r="L84" s="2"/>
+      <c r="M84" s="2"/>
+      <c r="N84" s="2"/>
+      <c r="O84" s="2"/>
+      <c r="P84" s="2"/>
+      <c r="Q84" s="2"/>
+      <c r="R84" s="2"/>
+      <c r="S84" s="2"/>
+      <c r="T84" s="2"/>
+      <c r="U84" s="2"/>
+      <c r="V84" s="2"/>
+      <c r="W84" s="2"/>
+      <c r="X84" s="2"/>
+      <c r="Y84" s="2"/>
+      <c r="Z84" s="2"/>
+    </row>
+    <row r="85" spans="1:26">
+      <c r="A85" s="2"/>
+      <c r="B85" s="2"/>
+      <c r="C85" s="2"/>
+      <c r="D85" s="2"/>
+      <c r="E85" s="2"/>
+      <c r="F85" s="2"/>
+      <c r="G85" s="2"/>
+      <c r="H85" s="2"/>
+      <c r="I85" s="2"/>
+      <c r="J85" s="2"/>
+      <c r="K85" s="2"/>
+      <c r="L85" s="2"/>
+      <c r="M85" s="2"/>
+      <c r="N85" s="2"/>
+      <c r="O85" s="2"/>
+      <c r="P85" s="2"/>
+      <c r="Q85" s="2"/>
+      <c r="R85" s="2"/>
+      <c r="S85" s="2"/>
+      <c r="T85" s="2"/>
+      <c r="U85" s="2"/>
+      <c r="V85" s="2"/>
+      <c r="W85" s="2"/>
+      <c r="X85" s="2"/>
+      <c r="Y85" s="2"/>
+      <c r="Z85" s="2"/>
+    </row>
+    <row r="86" spans="1:26">
+      <c r="A86" s="2"/>
+      <c r="B86" s="2"/>
+      <c r="C86" s="2"/>
+      <c r="D86" s="2"/>
+      <c r="E86" s="2"/>
+      <c r="F86" s="2"/>
+      <c r="G86" s="2"/>
+      <c r="H86" s="2"/>
+      <c r="I86" s="2"/>
+      <c r="J86" s="2"/>
+      <c r="K86" s="2"/>
+      <c r="L86" s="2"/>
+      <c r="M86" s="2"/>
+      <c r="N86" s="2"/>
+      <c r="O86" s="2"/>
+      <c r="P86" s="2"/>
+      <c r="Q86" s="2"/>
+      <c r="R86" s="2"/>
+      <c r="S86" s="2"/>
+      <c r="T86" s="2"/>
+      <c r="U86" s="2"/>
+      <c r="V86" s="2"/>
+      <c r="W86" s="2"/>
+      <c r="X86" s="2"/>
+      <c r="Y86" s="2"/>
+      <c r="Z86" s="2"/>
+    </row>
+    <row r="87" spans="1:26">
+      <c r="A87" s="2"/>
+      <c r="B87" s="2"/>
+      <c r="C87" s="2"/>
+      <c r="D87" s="2"/>
+      <c r="E87" s="2"/>
+      <c r="F87" s="2"/>
+      <c r="G87" s="2"/>
+      <c r="H87" s="2"/>
+      <c r="I87" s="2"/>
+      <c r="J87" s="2"/>
+      <c r="K87" s="2"/>
+      <c r="L87" s="2"/>
+      <c r="M87" s="2"/>
+      <c r="N87" s="2"/>
+      <c r="O87" s="2"/>
+      <c r="P87" s="2"/>
+      <c r="Q87" s="2"/>
+      <c r="R87" s="2"/>
+      <c r="S87" s="2"/>
+      <c r="T87" s="2"/>
+      <c r="U87" s="2"/>
+      <c r="V87" s="2"/>
+      <c r="W87" s="2"/>
+      <c r="X87" s="2"/>
+      <c r="Y87" s="2"/>
+      <c r="Z87" s="2"/>
+    </row>
+    <row r="88" spans="1:26">
+      <c r="A88" s="2"/>
+      <c r="B88" s="2"/>
+      <c r="C88" s="2"/>
+      <c r="D88" s="2"/>
+      <c r="E88" s="2"/>
+      <c r="F88" s="2"/>
+      <c r="G88" s="2"/>
+      <c r="H88" s="2"/>
+      <c r="I88" s="2"/>
+      <c r="J88" s="2"/>
+      <c r="K88" s="2"/>
+      <c r="L88" s="2"/>
+      <c r="M88" s="2"/>
+      <c r="N88" s="2"/>
+      <c r="O88" s="2"/>
+      <c r="P88" s="2"/>
+      <c r="Q88" s="2"/>
+      <c r="R88" s="2"/>
+      <c r="S88" s="2"/>
+      <c r="T88" s="2"/>
+      <c r="U88" s="2"/>
+      <c r="V88" s="2"/>
+      <c r="W88" s="2"/>
+      <c r="X88" s="2"/>
+      <c r="Y88" s="2"/>
+      <c r="Z88" s="2"/>
+    </row>
+    <row r="89" spans="1:26">
+      <c r="A89" s="2"/>
+      <c r="B89" s="2"/>
+      <c r="C89" s="2"/>
+      <c r="D89" s="2"/>
+      <c r="E89" s="2"/>
+      <c r="F89" s="2"/>
+      <c r="G89" s="2"/>
+      <c r="H89" s="2"/>
+      <c r="I89" s="2"/>
+      <c r="J89" s="2"/>
+      <c r="K89" s="2"/>
+      <c r="L89" s="2"/>
+      <c r="M89" s="2"/>
+      <c r="N89" s="2"/>
+      <c r="O89" s="2"/>
+      <c r="P89" s="2"/>
+      <c r="Q89" s="2"/>
+      <c r="R89" s="2"/>
+      <c r="S89" s="2"/>
+      <c r="T89" s="2"/>
+      <c r="U89" s="2"/>
+      <c r="V89" s="2"/>
+      <c r="W89" s="2"/>
+      <c r="X89" s="2"/>
+      <c r="Y89" s="2"/>
+      <c r="Z89" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Align raw coal catalog labels with TTCO stock data
</commit_message>
<xml_diff>
--- a/public/data/DS_kho_than_va_ty_khoi.xlsx
+++ b/public/data/DS_kho_than_va_ty_khoi.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OSC\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98A35D9A-9916-4A93-AAAD-714BD48C0750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D5CD23-267B-4EDC-B569-5984B74262E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -129,9 +129,6 @@
     <t>PX Tuyển than 2</t>
   </si>
   <si>
-    <t>Nguyên khai / Cám đá</t>
-  </si>
-  <si>
     <t>stt</t>
   </si>
   <si>
@@ -189,9 +186,6 @@
     <t>Cục xô 1C</t>
   </si>
   <si>
-    <t>Nguyên khai</t>
-  </si>
-  <si>
     <t>Đá thải</t>
   </si>
   <si>
@@ -303,12 +297,6 @@
     <t>Nhập khẩu / Bùn tuyển 3A</t>
   </si>
   <si>
-    <t>Cám đá / Nguyên khai</t>
-  </si>
-  <si>
-    <t>Nguyên khai / Cục don 8C</t>
-  </si>
-  <si>
     <t>Cám 6a.1 / Cục don 8C</t>
   </si>
   <si>
@@ -327,9 +315,6 @@
     <t>Cám 5a.1 / Cám 5a.14</t>
   </si>
   <si>
-    <t>Nguyên khai / Cám đá / Cám 6A.1 (sấy)</t>
-  </si>
-  <si>
     <t>Cám 3c.1</t>
   </si>
   <si>
@@ -349,6 +334,21 @@
   </si>
   <si>
     <t>Cám 8C</t>
+  </si>
+  <si>
+    <t>Cám đá / Than nguyên khai</t>
+  </si>
+  <si>
+    <t>Than nguyên khai / Cám đá</t>
+  </si>
+  <si>
+    <t>Than nguyên khai / Cám đá / Cám 6A.1 (sấy)</t>
+  </si>
+  <si>
+    <t>Than nguyên khai / Cục don 8C</t>
+  </si>
+  <si>
+    <t>Than nguyên khai</t>
   </si>
 </sst>
 </file>
@@ -691,13 +691,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -728,7 +728,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C2" s="5">
         <v>50.618279569892472</v>
@@ -737,7 +737,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -765,7 +765,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C3" s="5">
         <v>76.666666666666657</v>
@@ -774,7 +774,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -802,7 +802,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C4" s="5">
         <v>75.053763440860209</v>
@@ -811,7 +811,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -839,7 +839,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C5" s="5">
         <v>85.107526881720418</v>
@@ -848,7 +848,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -876,7 +876,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C6" s="5">
         <v>75.134408602150529</v>
@@ -885,7 +885,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -913,7 +913,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C7" s="5">
         <v>48.198924731182792</v>
@@ -922,7 +922,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -950,7 +950,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C8" s="5">
         <v>161.93548387096774</v>
@@ -959,7 +959,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -987,7 +987,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C9" s="5">
         <v>167.44623655913978</v>
@@ -996,7 +996,7 @@
         <v>37.200000000000003</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -1024,7 +1024,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C10" s="5">
         <v>229.70101309612059</v>
@@ -1033,7 +1033,7 @@
         <v>40.47</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
@@ -1061,7 +1061,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C11" s="5">
         <v>192.76006918705215</v>
@@ -1070,7 +1070,7 @@
         <v>40.47</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -1098,7 +1098,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C12" s="5">
         <v>141.19100568322213</v>
@@ -1107,7 +1107,7 @@
         <v>40.47</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -1135,7 +1135,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C13" s="5">
         <v>97.776130467012607</v>
@@ -1144,7 +1144,7 @@
         <v>40.47</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -1172,7 +1172,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C14" s="5">
         <v>69.360019767729185</v>
@@ -1181,7 +1181,7 @@
         <v>40.47</v>
       </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -1209,7 +1209,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C15" s="5">
         <v>68.668149246355327</v>
@@ -1218,7 +1218,7 @@
         <v>40.47</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1246,7 +1246,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C16" s="5">
         <v>130.9612058314801</v>
@@ -1255,7 +1255,7 @@
         <v>40.47</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1283,7 +1283,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C17" s="5">
         <v>114.22330097087378</v>
@@ -1292,7 +1292,7 @@
         <v>41.2</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1320,7 +1320,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C18" s="5">
         <v>286.09223300970871</v>
@@ -1329,7 +1329,7 @@
         <v>41.2</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1357,7 +1357,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C19" s="5">
         <v>81.626213592233</v>
@@ -1366,7 +1366,7 @@
         <v>41.2</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1394,7 +1394,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C20" s="5">
         <v>55.194174757281552</v>
@@ -1403,7 +1403,7 @@
         <v>41.2</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1431,7 +1431,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C21" s="5">
         <v>217.40291262135921</v>
@@ -1440,7 +1440,7 @@
         <v>41.2</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1468,7 +1468,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C22" s="5">
         <v>66.50485436893203</v>
@@ -1477,7 +1477,7 @@
         <v>41.2</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1505,7 +1505,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C23" s="5">
         <v>101.96601941747572</v>
@@ -1514,7 +1514,7 @@
         <v>41.2</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1542,7 +1542,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C24" s="5">
         <v>132.27011494252875</v>
@@ -1551,7 +1551,7 @@
         <v>34.799999999999997</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1579,7 +1579,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C25" s="5">
         <v>144.10919540229887</v>
@@ -1588,7 +1588,7 @@
         <v>34.799999999999997</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1616,7 +1616,7 @@
         <v>26</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C26" s="5">
         <v>134.77011494252875</v>
@@ -1625,7 +1625,7 @@
         <v>34.799999999999997</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1650,10 +1650,10 @@
     </row>
     <row r="27" spans="1:25">
       <c r="A27" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C27" s="6">
         <v>92.205542725173203</v>
@@ -1662,7 +1662,7 @@
         <v>34.64</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1687,10 +1687,10 @@
     </row>
     <row r="28" spans="1:25">
       <c r="A28" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C28" s="6">
         <v>109.06478578892371</v>
@@ -1699,7 +1699,7 @@
         <v>38.28</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -1724,10 +1724,10 @@
     </row>
     <row r="29" spans="1:25">
       <c r="A29" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C29" s="6">
         <v>108.76259798432251</v>
@@ -1736,7 +1736,7 @@
         <v>35.72</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -1761,10 +1761,10 @@
     </row>
     <row r="30" spans="1:25">
       <c r="A30" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C30" s="6">
         <v>108.34141610087293</v>
@@ -1773,7 +1773,7 @@
         <v>41.24</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -1801,7 +1801,7 @@
         <v>27</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C31" s="6">
         <v>194.60619062212686</v>
@@ -1810,7 +1810,7 @@
         <v>32.630000000000003</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -1838,7 +1838,7 @@
         <v>28</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C32" s="6">
         <v>118.97027275513331</v>
@@ -1847,7 +1847,7 @@
         <v>32.630000000000003</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -1884,7 +1884,7 @@
         <v>36.409999999999997</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -1909,10 +1909,10 @@
     </row>
     <row r="34" spans="1:25">
       <c r="A34" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C34" s="6">
         <v>110</v>
@@ -1921,7 +1921,7 @@
         <v>60</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -1946,10 +1946,10 @@
     </row>
     <row r="35" spans="1:25">
       <c r="A35" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C35" s="6">
         <v>227.33438842414651</v>
@@ -1958,7 +1958,7 @@
         <v>44.23</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
@@ -1983,10 +1983,10 @@
     </row>
     <row r="36" spans="1:25">
       <c r="A36" s="2" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C36" s="6">
         <v>150.87445346658336</v>
@@ -1995,7 +1995,7 @@
         <v>64.040000000000006</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -2020,10 +2020,10 @@
     </row>
     <row r="37" spans="1:25">
       <c r="A37" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C37" s="6">
         <v>292.70999999999998</v>
@@ -2032,7 +2032,7 @@
         <v>138.3519524443989</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -2057,10 +2057,10 @@
     </row>
     <row r="38" spans="1:25">
       <c r="A38" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C38" s="6">
         <v>191.39066863808117</v>
@@ -2069,7 +2069,7 @@
         <v>121.74</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -2094,10 +2094,10 @@
     </row>
     <row r="39" spans="1:25">
       <c r="A39" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C39" s="6">
         <v>189.93333333333334</v>
@@ -2106,7 +2106,7 @@
         <v>75</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -2131,10 +2131,10 @@
     </row>
     <row r="40" spans="1:25">
       <c r="A40" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C40" s="6">
         <v>210.89831909616976</v>
@@ -2143,7 +2143,7 @@
         <v>145.16</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -2168,10 +2168,10 @@
     </row>
     <row r="41" spans="1:25">
       <c r="A41" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C41" s="6">
         <v>214.11</v>
@@ -2180,7 +2180,7 @@
         <v>39.29288683387044</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
@@ -2205,10 +2205,10 @@
     </row>
     <row r="42" spans="1:25">
       <c r="A42" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C42" s="6">
         <v>182.01</v>
@@ -2217,7 +2217,7 @@
         <v>32.531179605516179</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -2242,10 +2242,10 @@
     </row>
     <row r="43" spans="1:25">
       <c r="A43" s="2" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C43" s="5">
         <v>267.51</v>
@@ -2254,7 +2254,7 @@
         <v>96.830025045792681</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
@@ -2279,10 +2279,10 @@
     </row>
     <row r="44" spans="1:25">
       <c r="A44" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C44" s="5">
         <v>148.08000000000001</v>
@@ -2291,7 +2291,7 @@
         <v>87.655321447866015</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>90</v>
+        <v>103</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -2316,10 +2316,10 @@
     </row>
     <row r="45" spans="1:25">
       <c r="A45" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C45" s="7">
         <v>192.38</v>
@@ -2328,15 +2328,15 @@
         <v>37.010084208337666</v>
       </c>
       <c r="E45" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:25">
       <c r="A46" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C46" s="6">
         <v>72.95</v>
@@ -2345,15 +2345,15 @@
         <v>60.137080191912268</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="47" spans="1:25">
       <c r="A47" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C47" s="6">
         <v>151.69999999999999</v>
@@ -2362,7 +2362,7 @@
         <v>45.484508899143052</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
@@ -3737,13 +3737,13 @@
   <sheetData>
     <row r="1" spans="1:26" ht="15">
       <c r="A1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -3774,7 +3774,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C2" s="3">
         <v>0.85117120418848147</v>
@@ -3808,7 +3808,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C3" s="3">
         <v>0.87113298429319397</v>
@@ -3842,7 +3842,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C4" s="3">
         <v>0.87776293193717259</v>
@@ -3876,7 +3876,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C5" s="3">
         <v>0.90840251366120195</v>
@@ -3910,7 +3910,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C6" s="3">
         <v>0.92027049180327902</v>
@@ -3944,7 +3944,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C7" s="3">
         <v>0.93945989071038305</v>
@@ -3978,7 +3978,7 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" s="3">
         <v>0.97699038251366144</v>
@@ -4012,7 +4012,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C9" s="3">
         <v>0.98199999999999998</v>
@@ -4046,7 +4046,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="3">
         <v>1.01316721311475</v>
@@ -4080,7 +4080,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C11" s="3">
         <v>1.01</v>
@@ -4114,7 +4114,7 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C12" s="3">
         <v>1.1045441530054649</v>
@@ -4148,7 +4148,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C13" s="3">
         <v>1.125</v>
@@ -4182,7 +4182,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="3">
         <v>1.0953590163934399</v>
@@ -4216,7 +4216,7 @@
         <v>14</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="3">
         <v>1.1842624043715826</v>
@@ -4250,7 +4250,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C16" s="3">
         <v>1.1512852459016401</v>
@@ -4284,7 +4284,7 @@
         <v>16</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C17" s="3">
         <v>1.1783234972677601</v>
@@ -4318,7 +4318,7 @@
         <v>17</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C18" s="3">
         <v>1.2069924590163925</v>
@@ -4352,7 +4352,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>51</v>
+        <v>104</v>
       </c>
       <c r="C19" s="3">
         <v>1.22525</v>
@@ -4386,7 +4386,7 @@
         <v>19</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C20" s="3">
         <v>0.93252816753926737</v>
@@ -4420,7 +4420,7 @@
         <v>20</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C21" s="3">
         <v>1.2562172631578901</v>
@@ -4454,7 +4454,7 @@
         <v>21</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="C22" s="3">
         <v>1.2350000000000001</v>
@@ -4488,7 +4488,7 @@
         <v>22</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C23" s="3">
         <v>1.26</v>
@@ -4522,7 +4522,7 @@
         <v>23</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="C24" s="3">
         <v>1.2649999999999999</v>
@@ -4556,7 +4556,7 @@
         <v>24</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="C25" s="3">
         <v>1.3049999999999999</v>
@@ -4590,7 +4590,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C26" s="3">
         <v>1.33</v>
@@ -4624,7 +4624,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="C27" s="3">
         <v>1.4019999999999999</v>
@@ -4658,7 +4658,7 @@
         <v>27</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C28" s="3">
         <v>1.3766666666666667</v>
@@ -4692,7 +4692,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C29" s="3">
         <v>1.2583689423076949</v>
@@ -4726,7 +4726,7 @@
         <v>29</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C30" s="3">
         <v>0.97824999999999995</v>
@@ -4760,7 +4760,7 @@
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C31" s="3">
         <v>1.5920000000000001</v>

</xml_diff>